<commit_message>
change some fields of certificates
</commit_message>
<xml_diff>
--- a/examples/excel_examples/federation-membership.xlsx
+++ b/examples/excel_examples/federation-membership.xlsx
@@ -186,7 +186,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">federation</t>
   </si>
@@ -252,6 +252,9 @@
   </si>
   <si>
     <t xml:space="preserve">Barcelona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A555557</t>
   </si>
   <si>
     <t xml:space="preserve">Full</t>
@@ -622,17 +625,20 @@
       <c r="H2" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="I2" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="J2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M2" s="6" t="n">
         <v>44928</v>
       </c>
       <c r="N2" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R2" s="6" t="n">
         <v>45292</v>

</xml_diff>